<commit_message>
Re-run the component notebooks and regenerate the figures
Sweeps in the pipeline re-execution sitting in the working tree: the
component notebooks for the Peninsula, EAIS, Greenland, glaciers, WAIS,
the summation and the forecast, the 46 figures that follow from them, the
results-figures notebook, the dataset inventory and the notebook audit
notes.

The results-figures notebook retains the changes made alongside this
work, so the regenerated Fig. 2 draws its callouts from the sample
probabilities and carries no slow-WAIS star, and Fig. 4b shows shares of
the 90% credible interval rather than variance fractions.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/slr_forecast/data/dataset_inventory.xlsx
+++ b/slr_forecast/data/dataset_inventory.xlsx
@@ -1241,7 +1241,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1972–2023 (observations from 1986)</t>
+          <t>1986–2023</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Values before 1986 are from the Kjeldsen et al. (2015) reconstruction. Shares raw data with Mouginot et al. (2019).</t>
+          <t>Shares raw data with Mouginot et al. (2019).</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>EAIS, Peninsula: comparison in component-notebook figures</t>
+          <t>EAIS, Peninsula: comparison in component-notebook figures; RCP2.6 runs (exp07) compared with SSP1-2.6 and RCP8.5 runs (exp05, exp06, exp08) with SSP5-8.5</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Rebased to 2000.</t>
+          <t>Standard melt parameterization, medium ocean sensitivity, no ice-shelf collapse. Rebased to 2000.</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Binds in 0.2% of SSP5-8.5 samples at 2100.</t>
+          <t>Binds in 0.1% of SSP5-8.5 samples at 2100.</t>
         </is>
       </c>
     </row>

</xml_diff>